<commit_message>
Updated catalog, change the structure in generate.py the product code before validation. admin folder is going to commited first time
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="139">
   <si>
     <t>Product Code</t>
   </si>
@@ -46,6 +46,9 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Image File</t>
+  </si>
+  <si>
     <t>ABT-001</t>
   </si>
   <si>
@@ -163,6 +166,12 @@
     <t>ABT-039</t>
   </si>
   <si>
+    <t>ABT-040</t>
+  </si>
+  <si>
+    <t>ABT-041</t>
+  </si>
+  <si>
     <t>Soaps</t>
   </si>
   <si>
@@ -187,6 +196,12 @@
     <t>Miscellaneous</t>
   </si>
   <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
     <t>Turkish Soap</t>
   </si>
   <si>
@@ -238,7 +253,7 @@
     <t>Tissue Paper (Clean)</t>
   </si>
   <si>
-    <t>LaSafety Razor</t>
+    <t>Lady Safety Razor</t>
   </si>
   <si>
     <t>Sensitive Toothbrush</t>
@@ -283,7 +298,7 @@
     <t>Khansama (Gol)</t>
   </si>
   <si>
-    <t>USIRooyal Cards (Plastic)</t>
+    <t>USA Royal Cards (Plastic)</t>
   </si>
   <si>
     <t>Paradise Jaali (30g)</t>
@@ -304,6 +319,12 @@
     <t>Golden Cards</t>
   </si>
   <si>
+    <t>Card1</t>
+  </si>
+  <si>
+    <t>brought up</t>
+  </si>
+  <si>
     <t>Carton (48 pcs)</t>
   </si>
   <si>
@@ -367,7 +388,7 @@
     <t>Carton (576 pcs)</t>
   </si>
   <si>
-    <t>Carton (100 rolls x 12 pcs = 1200 pcs</t>
+    <t>Carton (100 rolls)</t>
   </si>
   <si>
     <t>Packet (24 pcs)</t>
@@ -379,6 +400,12 @@
     <t>Carton (6 boxes x 20 pcs = 120 pcs)</t>
   </si>
   <si>
+    <t>13 packets</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
     <t>Confirm pack size with supplier</t>
   </si>
   <si>
@@ -395,6 +422,15 @@
   </si>
   <si>
     <t>Price is per roll; each roll cuts into ~12 pieces</t>
+  </si>
+  <si>
+    <t>nice product</t>
+  </si>
+  <si>
+    <t>Card1.png</t>
+  </si>
+  <si>
+    <t>brought_up.png</t>
   </si>
 </sst>
 </file>
@@ -752,10 +788,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -786,19 +822,22 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E2">
         <v>48</v>
@@ -810,21 +849,24 @@
         <v>52.0833333333333</v>
       </c>
       <c r="H2">
-        <v>62.0833333333333</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="E3">
         <v>144</v>
@@ -836,21 +878,24 @@
         <v>7.63888888888889</v>
       </c>
       <c r="H3">
-        <v>17.6388888888889</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E4">
         <v>12</v>
@@ -862,21 +907,24 @@
         <v>27.5</v>
       </c>
       <c r="H4">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E5">
         <v>12</v>
@@ -888,21 +936,24 @@
         <v>27.5</v>
       </c>
       <c r="H5">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -914,21 +965,24 @@
         <v>37.5</v>
       </c>
       <c r="H6">
-        <v>47.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -940,24 +994,27 @@
         <v>54.1666666666667</v>
       </c>
       <c r="H7">
-        <v>64.1666666666667</v>
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D8" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E8">
         <v>12</v>
@@ -969,21 +1026,24 @@
         <v>15.8333333333333</v>
       </c>
       <c r="H8">
-        <v>25.8333333333333</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -995,21 +1055,24 @@
         <v>11</v>
       </c>
       <c r="H9">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D10" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E10">
         <v>10</v>
@@ -1021,24 +1084,27 @@
         <v>19.5</v>
       </c>
       <c r="H10">
-        <v>29.5</v>
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D11" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E11">
         <v>12</v>
@@ -1050,21 +1116,24 @@
         <v>23.3333333333333</v>
       </c>
       <c r="H11">
-        <v>33.3333333333333</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D12" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E12">
         <v>20</v>
@@ -1076,21 +1145,24 @@
         <v>46.5</v>
       </c>
       <c r="H12">
-        <v>56.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E13">
         <v>384</v>
@@ -1102,21 +1174,24 @@
         <v>14.3229166666667</v>
       </c>
       <c r="H13">
-        <v>24.3229166666667</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D14" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="E14">
         <v>24</v>
@@ -1128,24 +1203,27 @@
         <v>28.3333333333333</v>
       </c>
       <c r="H14">
-        <v>38.3333333333333</v>
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -1157,21 +1235,24 @@
         <v>30</v>
       </c>
       <c r="H15">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D16" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="E16">
         <v>600</v>
@@ -1183,21 +1264,24 @@
         <v>5</v>
       </c>
       <c r="H16">
-        <v>15</v>
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="E17">
         <v>60</v>
@@ -1209,21 +1293,24 @@
         <v>4.33333333333333</v>
       </c>
       <c r="H17">
-        <v>14.3333333333333</v>
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D18" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="E18">
         <v>60</v>
@@ -1235,24 +1322,27 @@
         <v>103.333333333333</v>
       </c>
       <c r="H18">
-        <v>113.333333333333</v>
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
       </c>
       <c r="J18" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D19" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E19">
         <v>6</v>
@@ -1264,21 +1354,24 @@
         <v>8.33333333333333</v>
       </c>
       <c r="H19">
-        <v>18.3333333333333</v>
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D20" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E20">
         <v>12</v>
@@ -1290,21 +1383,24 @@
         <v>25</v>
       </c>
       <c r="H20">
-        <v>35</v>
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E21">
         <v>12</v>
@@ -1316,21 +1412,24 @@
         <v>91.6666666666667</v>
       </c>
       <c r="H21">
-        <v>101.666666666667</v>
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D22" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E22">
         <v>12</v>
@@ -1342,21 +1441,24 @@
         <v>76.6666666666667</v>
       </c>
       <c r="H22">
-        <v>86.6666666666667</v>
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D23" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -1368,21 +1470,24 @@
         <v>83</v>
       </c>
       <c r="H23">
-        <v>93</v>
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D24" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E24">
         <v>12</v>
@@ -1394,21 +1499,24 @@
         <v>37.5</v>
       </c>
       <c r="H24">
-        <v>47.5</v>
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D25" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E25">
         <v>1000</v>
@@ -1420,21 +1528,24 @@
         <v>3.1</v>
       </c>
       <c r="H25">
-        <v>13.1</v>
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D26" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E26">
         <v>12</v>
@@ -1446,24 +1557,27 @@
         <v>250</v>
       </c>
       <c r="H26">
-        <v>260</v>
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
       </c>
       <c r="J26" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C27" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D27" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="E27">
         <v>576</v>
@@ -1475,21 +1589,24 @@
         <v>8.680555555555561</v>
       </c>
       <c r="H27">
-        <v>18.6805555555556</v>
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C28" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D28" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="E28">
         <v>576</v>
@@ -1501,21 +1618,24 @@
         <v>12.1527777777778</v>
       </c>
       <c r="H28">
-        <v>22.1527777777778</v>
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C29" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D29" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="E29">
         <v>576</v>
@@ -1527,21 +1647,24 @@
         <v>5.20833333333333</v>
       </c>
       <c r="H29">
-        <v>15.2083333333333</v>
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C30" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D30" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="E30">
         <v>576</v>
@@ -1553,21 +1676,24 @@
         <v>16.4930555555556</v>
       </c>
       <c r="H30">
-        <v>26.4930555555556</v>
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C31" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D31" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="E31">
         <v>576</v>
@@ -1579,50 +1705,56 @@
         <v>11.2847222222222</v>
       </c>
       <c r="H31">
-        <v>21.2847222222222</v>
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D32" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="E32">
-        <v>1200</v>
+        <v>100</v>
       </c>
       <c r="F32">
         <v>4800</v>
       </c>
       <c r="G32">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="H32">
-        <v>14</v>
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
       </c>
       <c r="J32" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D33" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="E33">
         <v>24</v>
@@ -1634,21 +1766,24 @@
         <v>8.75</v>
       </c>
       <c r="H33">
-        <v>18.75</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C34" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D34" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="E34">
         <v>144</v>
@@ -1660,21 +1795,24 @@
         <v>131.944444444444</v>
       </c>
       <c r="H34">
-        <v>141.944444444444</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C35" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D35" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E35">
         <v>12</v>
@@ -1686,21 +1824,24 @@
         <v>29.1666666666667</v>
       </c>
       <c r="H35">
-        <v>39.1666666666667</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C36" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D36" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E36">
         <v>12</v>
@@ -1712,21 +1853,24 @@
         <v>26.6666666666667</v>
       </c>
       <c r="H36">
-        <v>36.6666666666667</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D37" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E37">
         <v>12</v>
@@ -1738,21 +1882,24 @@
         <v>14.1666666666667</v>
       </c>
       <c r="H37">
-        <v>24.1666666666667</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C38" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D38" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E38">
         <v>12</v>
@@ -1764,21 +1911,24 @@
         <v>10</v>
       </c>
       <c r="H38">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C39" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D39" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E39">
         <v>12</v>
@@ -1790,21 +1940,24 @@
         <v>8.75</v>
       </c>
       <c r="H39">
-        <v>18.75</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C40" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D40" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="E40">
         <v>120</v>
@@ -1816,7 +1969,77 @@
         <v>72.5</v>
       </c>
       <c r="H40">
-        <v>82.5</v>
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" t="s">
+        <v>60</v>
+      </c>
+      <c r="C41" t="s">
+        <v>101</v>
+      </c>
+      <c r="D41" t="s">
+        <v>128</v>
+      </c>
+      <c r="E41">
+        <v>145</v>
+      </c>
+      <c r="F41">
+        <v>789</v>
+      </c>
+      <c r="G41">
+        <v>67</v>
+      </c>
+      <c r="H41">
+        <v>12</v>
+      </c>
+      <c r="I41">
+        <v>16</v>
+      </c>
+      <c r="J41" t="s">
+        <v>136</v>
+      </c>
+      <c r="K41" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
+      <c r="A42" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" t="s">
+        <v>102</v>
+      </c>
+      <c r="D42" t="s">
+        <v>129</v>
+      </c>
+      <c r="E42">
+        <v>12</v>
+      </c>
+      <c r="F42">
+        <v>390</v>
+      </c>
+      <c r="G42">
+        <v>45</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="K42" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>